<commit_message>
update daily dashboard 2026-10-11
Backfill week 2026-10-05–11 from learning-planner exports; refresh weekly history and detail pages.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/每日输出/小短/郑州-小短-每日风灵不在线.xlsx
+++ b/每日输出/小短/郑州-小短-每日风灵不在线.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +35,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +55,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
   </fills>
@@ -80,12 +89,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -453,13 +474,1435 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:X14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>无数据</t>
+          <t>服务期</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>运营中心</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>分部</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>系统来源</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>学段</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>wehook_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>阶段</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>战队</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>日期</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>学习规划师姓名</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>学习规划师邮箱</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>推广产品</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>风灵在线率</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>不在线时段list</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>app在线率</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>app不在线时段list</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>pc在线率</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>pc不在线时段list</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>年级</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>老师姓名</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>销售邮箱</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>sys_source</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>学部</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>分组</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1688855425700511</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>李丹阳</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>lidanyang</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>李丹阳</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>lidanyang</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1688855001729445</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>李少辉</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>lishaohui</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>李少辉</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>lishaohui</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1688856042840562</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>wangcongyang</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>9,10,11,12,13</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>9,10,11,12,13</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>wangcongyang</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1688854397763628</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>李京哲</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>lijingzhe</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>李京哲</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>lijingzhe</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>1688854644796116</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>荆雅博</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>jingyabo</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>1</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>荆雅博</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>jingyabo</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>1688856227810743</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>陈湘茹</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>chenxiangru</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>陈湘茹</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>chenxiangru</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1688854619909919</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>刘栋辉</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>liudonghui</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>刘栋辉</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>liudonghui</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1688854426767496</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>杨喜菊</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>yangxiju</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>杨喜菊</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>yangxiju</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1688854876688129</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>王梦迪</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>wangmengdi01</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>王梦迪</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>wangmengdi01</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>1688854644796118</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>张昱莹</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>zhangyuying01</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>张昱莹</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>zhangyuying01</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1688858040865393</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>王欣冉</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>wangxinran</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>王欣冉</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>wangxinran</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1688858172724149</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>吕志恒</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>lvzhiheng</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>吕志恒</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>lvzhiheng</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>小短</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>20261009</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>郑州</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>短期班</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>小阶</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1688856448789579</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>全部</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>wuxiayan</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>低价课</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>wuxiayan</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>爱学</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>小短</t>
         </is>
       </c>
     </row>
@@ -474,7 +1917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R15"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -571,11 +2014,11 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -600,17 +2043,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>peifang</t>
+          <t>yangxiju</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>裴芳</t>
+          <t>杨喜菊</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -619,11 +2062,11 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+          <t>17</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -638,12 +2081,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>peifang</t>
+          <t>yangxiju</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>裴芳</t>
+          <t>杨喜菊</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -659,11 +2102,11 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -688,17 +2131,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>秦淑楠</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>lijingzhe</t>
+          <t>wangxinran</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>李京哲</t>
+          <t>王欣冉</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -721,12 +2164,12 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>lijingzhe</t>
+          <t>wangxinran</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>李京哲</t>
+          <t>王欣冉</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -742,11 +2185,11 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -776,12 +2219,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>wangmengdi01</t>
+          <t>lishaohui</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>王梦迪</t>
+          <t>李少辉</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -790,12 +2233,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -809,12 +2247,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>wangmengdi01</t>
+          <t>lishaohui</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>王梦迪</t>
+          <t>李少辉</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -830,11 +2268,11 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -859,17 +2297,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>秦淑楠</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>lishaohui</t>
+          <t>wuxiayan</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>李少辉</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -878,7 +2316,12 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -892,12 +2335,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>lishaohui</t>
+          <t>wuxiayan</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>李少辉</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -913,11 +2356,11 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -947,12 +2390,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>chenxiangru</t>
+          <t>lvzhiheng</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>陈湘茹</t>
+          <t>吕志恒</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -975,12 +2418,12 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>chenxiangru</t>
+          <t>lvzhiheng</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>陈湘茹</t>
+          <t>吕志恒</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -996,11 +2439,11 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1084,11 +2527,11 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1118,12 +2561,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>wangxinran</t>
+          <t>liudonghui</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>王欣冉</t>
+          <t>刘栋辉</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1132,12 +2575,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1151,12 +2589,12 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>wangxinran</t>
+          <t>liudonghui</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>王欣冉</t>
+          <t>刘栋辉</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1172,11 +2610,11 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1201,17 +2639,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>秦淑楠</t>
+          <t>仵夏炎</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>yangxiju</t>
+          <t>chenxiangru</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>杨喜菊</t>
+          <t>陈湘茹</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1234,12 +2672,12 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>yangxiju</t>
+          <t>chenxiangru</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>杨喜菊</t>
+          <t>陈湘茹</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -1255,11 +2693,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1284,17 +2722,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>jingyabo</t>
+          <t>lidanyang</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>荆雅博</t>
+          <t>李丹阳</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1303,12 +2741,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1322,12 +2755,12 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>jingyabo</t>
+          <t>lidanyang</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>荆雅博</t>
+          <t>李丹阳</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -1343,11 +2776,11 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1372,17 +2805,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>liudonghui</t>
+          <t>wangmengdi01</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>刘栋辉</t>
+          <t>王梦迪</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1410,12 +2843,12 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>liudonghui</t>
+          <t>wangmengdi01</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>刘栋辉</t>
+          <t>王梦迪</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -1431,11 +2864,11 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1460,17 +2893,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>秦淑楠</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>lvzhiheng</t>
+          <t>zhangyuying01</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>吕志恒</t>
+          <t>张昱莹</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1479,7 +2912,12 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
+        </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1493,12 +2931,12 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>lvzhiheng</t>
+          <t>zhangyuying01</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>吕志恒</t>
+          <t>张昱莹</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1514,11 +2952,11 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1548,12 +2986,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>wuxiayan</t>
+          <t>jingyabo</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>荆雅博</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1581,12 +3019,12 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>wuxiayan</t>
+          <t>jingyabo</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>仵夏炎</t>
+          <t>荆雅博</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1602,11 +3040,11 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>20260918</v>
+        <v>20261009</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1636,12 +3074,12 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>zhangyuying01</t>
+          <t>lijingzhe</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>张昱莹</t>
+          <t>李京哲</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1650,12 +3088,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>6,7,8,9,10,11,12,13,14,15,16,17,18,19,20,21,22,23</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1669,12 +3102,12 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>zhangyuying01</t>
+          <t>lijingzhe</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>张昱莹</t>
+          <t>李京哲</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1683,89 +3116,6 @@
         </is>
       </c>
       <c r="R14" t="inlineStr">
-        <is>
-          <t>小短</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>20260918</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>短期班</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>全部</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>郑州</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>秦淑楠</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>lidanyang</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>李丹阳</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>低价课</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>1</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>全年级</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>小学</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>lidanyang</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>李丹阳</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>爱学</t>
-        </is>
-      </c>
-      <c r="R15" t="inlineStr">
         <is>
           <t>小短</t>
         </is>
@@ -1782,7 +3132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1797,7 +3147,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>风灵在线未达标名单（小短）-9月20日（低价课）</t>
+          <t>风灵在线未达标名单（小短）-10月11日（低价课）</t>
         </is>
       </c>
     </row>
@@ -1836,6 +3186,192 @@
         <is>
           <t>个微在线率</t>
         </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>仵夏炎</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>荆雅博</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>0.6111111111111112</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>张昱莹</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>杨喜菊</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>王梦迪</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>小学</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>全年级</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>秦淑楠</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>王聪阳</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>0.7222222222222222</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>